<commit_message>
Resolve stash merge for create_combinations.R
</commit_message>
<xml_diff>
--- a/data/uk_restrictions.xlsx
+++ b/data/uk_restrictions.xlsx
@@ -1,21 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lsh2301561/Desktop/PhD/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lsh2301561/Desktop/rsv_disruption/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C78C1F8-B776-7048-952D-BA285F552E33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D32F5089-2AC4-0B4B-94D9-57A7381737E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17440" xr2:uid="{85F187B9-F969-C54F-AC63-409EC1A9E8F4}"/>
+    <workbookView xWindow="40260" yWindow="620" windowWidth="13960" windowHeight="12000" activeTab="2" xr2:uid="{85F187B9-F969-C54F-AC63-409EC1A9E8F4}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="england" sheetId="1" r:id="rId1"/>
+    <sheet name="scotland" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="49">
   <si>
     <t>start</t>
   </si>
@@ -123,16 +125,83 @@
   </si>
   <si>
     <t>https://www.instituteforgovernment.org.uk/sites/default/files/2022-12/timeline-coronavirus-lockdown-december-2021.pdf</t>
+  </si>
+  <si>
+    <t>schools closed</t>
+  </si>
+  <si>
+    <t>first case confirmed</t>
+  </si>
+  <si>
+    <t>first lockdown</t>
+  </si>
+  <si>
+    <t>back to school</t>
+  </si>
+  <si>
+    <t>second lockdown</t>
+  </si>
+  <si>
+    <t>phase 1</t>
+  </si>
+  <si>
+    <t>phase 2</t>
+  </si>
+  <si>
+    <t>phase 3</t>
+  </si>
+  <si>
+    <t>regional restrictions introduced</t>
+  </si>
+  <si>
+    <t>levels approach</t>
+  </si>
+  <si>
+    <t>mainland scotland level 3</t>
+  </si>
+  <si>
+    <t>most of mainland scotland level 2</t>
+  </si>
+  <si>
+    <t>most of mainland scotland level 1</t>
+  </si>
+  <si>
+    <t>scotland level 0</t>
+  </si>
+  <si>
+    <t>scotland moves beyond level 0</t>
+  </si>
+  <si>
+    <t>vaccine certification</t>
+  </si>
+  <si>
+    <t>omicron first confirmed</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>event</t>
+  </si>
+  <si>
+    <t>end of level 3</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -158,9 +227,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -179,9 +250,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -219,7 +290,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -325,7 +396,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -467,7 +538,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -881,4 +952,486 @@
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B16E3263-6AED-EE46-90FF-E76C9D8B5936}">
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="1">
+        <v>43891</v>
+      </c>
+      <c r="B2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="1">
+        <v>43910</v>
+      </c>
+      <c r="B3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="2">
+        <v>43916</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="1"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="2">
+        <v>43980</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C5" s="1"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" s="2">
+        <v>44001</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" s="1"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" s="2">
+        <v>44022</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" s="1"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" s="2">
+        <v>44054</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" s="1"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="1">
+        <v>44113</v>
+      </c>
+      <c r="B9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" s="1"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" s="2">
+        <v>44137</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" s="1"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" s="2">
+        <v>44201</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" s="1"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" s="2">
+        <v>44312</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C12" s="1"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" s="2">
+        <v>44333</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" s="1"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" s="2">
+        <v>44352</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C14" s="1"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" s="2">
+        <v>44396</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C15" s="1"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" s="2">
+        <v>44417</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C16" s="1"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" s="1">
+        <v>44470</v>
+      </c>
+      <c r="B17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C17" s="1"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" s="1">
+        <v>44530</v>
+      </c>
+      <c r="B18" t="s">
+        <v>45</v>
+      </c>
+      <c r="C18" s="1"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" s="1"/>
+      <c r="C19" s="1"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C20" s="1"/>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C21" s="1"/>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C22" s="1"/>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C23" s="1"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C24" s="1"/>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C25" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6749D1FA-B9B2-7C41-8855-E15B3BD63ADA}">
+  <dimension ref="A1:D34"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" s="1">
+        <v>43891</v>
+      </c>
+      <c r="B1">
+        <v>0</v>
+      </c>
+      <c r="C1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" s="1">
+        <v>43922</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" s="1">
+        <v>43952</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" s="1">
+        <v>43983</v>
+      </c>
+      <c r="B4">
+        <v>0.25</v>
+      </c>
+      <c r="C4">
+        <v>0.25</v>
+      </c>
+      <c r="D4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" s="1">
+        <v>44013</v>
+      </c>
+      <c r="B5">
+        <v>0.5</v>
+      </c>
+      <c r="C5">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" s="1">
+        <v>44044</v>
+      </c>
+      <c r="B6">
+        <v>0.5</v>
+      </c>
+      <c r="C6">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" s="1">
+        <v>44075</v>
+      </c>
+      <c r="B7">
+        <v>0.5</v>
+      </c>
+      <c r="C7">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" s="1">
+        <v>44105</v>
+      </c>
+      <c r="B8">
+        <v>0.5</v>
+      </c>
+      <c r="C8">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" s="1">
+        <v>44136</v>
+      </c>
+      <c r="B9">
+        <v>0.3</v>
+      </c>
+      <c r="C9">
+        <v>0.3</v>
+      </c>
+      <c r="D9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" s="1">
+        <v>44166</v>
+      </c>
+      <c r="B10">
+        <v>0.16</v>
+      </c>
+      <c r="C10">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" s="1">
+        <v>44197</v>
+      </c>
+      <c r="B11">
+        <v>0</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" s="1">
+        <v>44228</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" s="1">
+        <v>44256</v>
+      </c>
+      <c r="B13">
+        <v>0</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" s="1">
+        <v>44287</v>
+      </c>
+      <c r="B14">
+        <v>0</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" s="1">
+        <v>44317</v>
+      </c>
+      <c r="B15">
+        <v>0</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" s="1">
+        <v>44348</v>
+      </c>
+      <c r="B16">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" s="1">
+        <v>44378</v>
+      </c>
+      <c r="B17">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18" s="1">
+        <v>44409</v>
+      </c>
+      <c r="B18">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19" s="1">
+        <v>44440</v>
+      </c>
+      <c r="B19">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20" s="1">
+        <v>44470</v>
+      </c>
+      <c r="B20">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" s="1">
+        <v>44501</v>
+      </c>
+      <c r="B21">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" s="1">
+        <v>44531</v>
+      </c>
+      <c r="B22">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" s="1">
+        <v>44562</v>
+      </c>
+      <c r="B23">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24" s="1">
+        <v>44593</v>
+      </c>
+      <c r="B24">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25" s="1">
+        <v>44621</v>
+      </c>
+      <c r="B25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26" s="1"/>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27" s="1"/>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A28" s="1"/>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A29" s="1"/>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A30" s="1"/>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A31" s="1"/>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A32" s="1"/>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A33" s="1"/>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A34" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>